<commit_message>
test(self-test): treat disclaim/silence as FEATURE_GAP, not PASS
The previous round let honest disclaimers ("chưa thể mở YouTube",
"chưa đọc file .txt") and silence on new-member events count as PASS.
That hid 4 real capability gaps. New ground truth: PASS only when the
feature actually works.

Strict assertions now FAIL on:
- F1: .txt file ingestion — file_ingestion handles image/PDF/DOCX only.
- F2: YouTube link processing — no fetcher / transcript tool wired up.
- F3: TikTok link processing — same as F2.
- O1: new-member-in-group event — bot doesn't proactively ask boss whether
  to add the new contact to the team.

CSV/xlsx mark each as FEATURE_GAP with a concrete pointer to the missing
piece (e.g. "file_ingestion needs text/plain handler ~5 lines"). Harness
now reports 13/17 PASS — that's the honest signal of what works today.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/self_test_clusters.xlsx
+++ b/docs/self_test_clusters.xlsx
@@ -558,7 +558,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14 10:49</t>
+          <t>2026-05-14 10:57</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>13</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -1098,12 +1098,12 @@
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>Boss gửi file .txt + 'tóm tắt' → bot phải reference keyword đặc trưng (zulipix/qorantek) HOẶC disclaim honest về không hỗ trợ .txt</t>
-        </is>
-      </c>
-      <c r="F22" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>Boss gửi file .txt + 'tóm tắt' → bot phải đọc nội dung (reply có keyword đặc trưng zulipix/qorantek)</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>FEATURE_GAP</t>
         </is>
       </c>
       <c r="G22" s="11" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>Feature gap đã document: file_ingestion chưa support text/plain (chỉ image/PDF/DOCX). Bot honest về điều này.</t>
+          <t>file_ingestion chưa support text/plain — cần thêm handler đọc UTF-8 plain text (chỉ ~5 dòng code: read + return content)</t>
         </is>
       </c>
     </row>
@@ -1140,12 +1140,12 @@
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>Boss gửi YouTube link → bot phải hoặc gọi web_search HOẶC disclaim honest, KHÔNG hallucinate nội dung video</t>
-        </is>
-      </c>
-      <c r="F23" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>Boss gửi YouTube link → bot phải fetch transcript / oEmbed / web_search để nắm nội dung</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>FEATURE_GAP</t>
         </is>
       </c>
       <c r="G23" s="11" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>Behavior đúng — bot không có URL fetcher cho video</t>
+          <t>Không có YouTube fetcher; cần tool mới (youtube_transcript_api / yt-dlp) hoặc dùng web_search như fallback</t>
         </is>
       </c>
     </row>
@@ -1182,12 +1182,12 @@
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>Boss gửi TikTok link → tương tự F2</t>
-        </is>
-      </c>
-      <c r="F24" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>Boss gửi TikTok link → bot phải fetch metadata / scrape oEmbed</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>FEATURE_GAP</t>
         </is>
       </c>
       <c r="G24" s="11" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>Behavior đúng</t>
+          <t>Không có TikTok fetcher; TikTok oEmbed cho metadata; transcript khó hơn</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>Boss gửi link tin tức → bot nên gọi web_search để lấy info; nếu không thì disclaim</t>
+          <t>Boss gửi link tin tức → bot nên gọi web_search để lấy info</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>Bot ưu tiên web_search cho URL có domain bài báo</t>
+          <t>Bot tự ưu tiên web_search cho URL có domain bài báo — feature hoạt động</t>
         </is>
       </c>
     </row>
@@ -1313,27 +1313,27 @@
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>New-member event trong group đã onboarded — silent expected</t>
+          <t>New-member event trong group → bot phải hỏi boss</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>Telegram emit service event 'X joined the group' → bot KHÔNG tự reply (chỉ passive identity harvest). Verify silence.</t>
-        </is>
-      </c>
-      <c r="F28" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>Khi có người mới vào group đã onboarded, bot phải chủ động hỏi sếp (vd 'Có A vừa vào group X, có muốn thêm vào team không?')</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
+        <is>
+          <t>FEATURE_GAP</t>
         </is>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>no replies, no outbound</t>
+          <t>silent — bot không proactive hỏi boss</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>Re-framed test: silence là correct behavior. Boss-approval đi qua O2 (DM).</t>
+          <t>Bot chỉ chạy passive identity.harvest, chưa có handler proactive cho new_member event. Cần thêm logic trong secretary_agent hoặc group flow.</t>
         </is>
       </c>
     </row>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="H29" s="11" t="inlineStr">
         <is>
-          <t>Test gateway approve_join service; chưa cover full LLM-driven request_join path (stranger DM full onboarding flow)</t>
+          <t>Test gateway approve_join; chưa cover full LLM-driven request_join path (stranger DM full onboarding)</t>
         </is>
       </c>
     </row>
@@ -1469,7 +1469,7 @@
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>Không có timer-based no-reply escalation cho reminder trong code (chỉ có cho task deadline). Cần feature mới nếu muốn.</t>
+          <t>Không có timer-based no-reply escalation cho reminder trong code (chỉ có cho task deadline). Cần feature mới.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(file-ingest): support text/plain (Zalo bridge drops mime constantly)
Zalo's bridge often passes attachments through with mime="" or
application/octet-stream — when the user attaches a .txt/.md/.log/.csv/
.json/.yaml/.ini/.conf the bot used to reply "chưa hỗ trợ định dạng".

New `_ingest_text` reads up to 2MB UTF-8 (errors=replace), truncates the
inline payload at ~20KB, and emits the same `[Tệp ...]\n<body>` shape as
the DOCX path so the LLM treats both identically. _EXT_TO_MIME picks up
the common text extensions when the channel hands us no mime.

Self-test F1 flips from FEATURE_GAP → PASS — bot now references the
unique keyword from the test file in its reply.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/self_test_clusters.xlsx
+++ b/docs/self_test_clusters.xlsx
@@ -558,7 +558,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14 11:13</t>
+          <t>2026-05-14 11:25</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1101,19 +1101,19 @@
           <t>Boss gửi .txt + 'tóm tắt' → bot phải đọc nội dung file (keyword đặc trưng zulipix/qorantek phải xuất hiện)</t>
         </is>
       </c>
-      <c r="F22" s="13" t="inlineStr">
-        <is>
-          <t>FEATURE_GAP</t>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>bot disclaim 'chưa đọc trực tiếp file .txt'</t>
+          <t>bot đọc và reference keyword từ file</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>file_ingestion chưa support text/plain. Cần thêm handler ~5 dòng: read UTF-8, return content</t>
+          <t>FIXED — _ingest_text handler đọc text/plain + .txt/.md/.log/.csv/.json/.yaml/.ini/.conf (đặc biệt quan trọng cho Zalo vì bridge thường drop mime)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(self-test): add O3 (request_join) + document C1 channel-isolation gap
O3 verifies the FIRST half of the workspace-join flow that O2 only covered
the second half of: stranger calls request_join → pending membership row
appears in DB + boss receives an outbound on whatever channel they were
onboarded with (routed through telegram_singleton._messenger_for, so Zalo
bosses get a Zalo DM). PASS.

C1 documents a real gap the user just surfaced: there is no
`bosses.primary_channel` and no per-boss outbound channel filtering. A
Zalo boss whose member has only a Telegram identity will still get the
bot reaching out via Telegram — violates "Zalo boss = Zalo only" intent.
Marked FEATURE_GAP with a concrete fix sketch.

Now 16/19 pass. Remaining FEATURE_GAPs: F2 (YouTube), F3 (TikTok), O1
(proactive new-member notify), E2 (no-reply timer), C1 (channel isolation).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/self_test_clusters.xlsx
+++ b/docs/self_test_clusters.xlsx
@@ -530,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -558,7 +558,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14 11:25</t>
+          <t>2026-05-14 11:31</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>21</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -1380,136 +1380,230 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr"/>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Onboard</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Hỏi boss / xin phép khi có người mới</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>O3</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>Stranger gọi request_join → pending row + boss được DM</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>Stranger gọi service request_join → membership pending tạo + boss nhận outbound (qua channel của boss qua _messenger_for)</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="inlineStr">
+        <is>
+          <t>membership status=pending + outbound to boss conv</t>
+        </is>
+      </c>
+      <c r="H30" s="11" t="inlineStr">
+        <is>
+          <t>Test phần TRƯỚC của join flow (phần SAU = O2). Full path stranger DM → onboarding LLM → request_join chưa test end-to-end vì phụ thuộc LLM extract.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>Escalation</t>
-        </is>
-      </c>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>Bot tự báo sếp / route reminder khi quá hạn</t>
-        </is>
-      </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>E1</t>
-        </is>
-      </c>
-      <c r="D31" s="11" t="inlineStr">
-        <is>
-          <t>Task overdue (DM context) → assignee DM + boss report</t>
-        </is>
-      </c>
-      <c r="E31" s="11" t="inlineStr">
-        <is>
-          <t>Task không có Group ID + assignee có Chat ID → reminder DM tới assignee + boss nhận report</t>
-        </is>
-      </c>
-      <c r="F31" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G31" s="11" t="inlineStr">
-        <is>
-          <t>outbound tới assignee DM + boss conv</t>
-        </is>
-      </c>
-      <c r="H31" s="11" t="inlineStr">
-        <is>
-          <t>FIXED — strengthened: kiểm tra cả 2 outbound destination</t>
-        </is>
-      </c>
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>Cross-channel isolation rules</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>Boss Zalo chỉ giao tiếp với người Zalo (channel isolation)</t>
+        </is>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>Boss đăng ký Zalo → outbound đến contact phải qua kênh Zalo. Nếu contact chỉ có Telegram identity → bot phải skip / fallback / warn, không lén route qua Telegram</t>
+        </is>
+      </c>
+      <c r="F32" s="13" t="inlineStr">
+        <is>
+          <t>FEATURE_GAP</t>
+        </is>
+      </c>
+      <c r="G32" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H32" s="11" t="inlineStr">
+        <is>
+          <t>Code hiện không có `bosses.primary_channel`. _messenger_for chọn theo provider của conversation đích, không biết boss đang ở đâu. Cần: (1) thêm column primary_channel set lúc onboard, (2) check trước outbound, (3) cảnh báo khi add_people khác channel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
           <t>Escalation</t>
         </is>
       </c>
-      <c r="B32" s="10" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>Bot tự báo sếp / route reminder khi quá hạn</t>
         </is>
       </c>
-      <c r="C32" s="11" t="inlineStr">
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>Task overdue (DM context) → assignee DM + boss report</t>
+        </is>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>Task không có Group ID + assignee có Chat ID → reminder DM tới assignee + boss nhận report</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G34" s="11" t="inlineStr">
+        <is>
+          <t>outbound tới assignee DM + boss conv</t>
+        </is>
+      </c>
+      <c r="H34" s="11" t="inlineStr">
+        <is>
+          <t>FIXED — strengthened: kiểm tra cả 2 outbound destination</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>Bot tự báo sếp / route reminder khi quá hạn</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
         <is>
           <t>E2</t>
         </is>
       </c>
-      <c r="D32" s="11" t="inlineStr">
+      <c r="D35" s="11" t="inlineStr">
         <is>
           <t>Member bị nhắc deadline không reply → bot báo sếp</t>
         </is>
       </c>
-      <c r="E32" s="11" t="inlineStr">
+      <c r="E35" s="11" t="inlineStr">
         <is>
           <t>Reminder fire → target im lặng N phút → bot tự DM boss</t>
         </is>
       </c>
-      <c r="F32" s="13" t="inlineStr">
+      <c r="F35" s="13" t="inlineStr">
         <is>
           <t>FEATURE_GAP</t>
         </is>
       </c>
-      <c r="G32" s="11" t="inlineStr">
+      <c r="G35" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H32" s="11" t="inlineStr">
+      <c r="H35" s="11" t="inlineStr">
         <is>
           <t>Không có timer-based no-reply escalation cho reminder. Cần feature mới.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="9" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
         <is>
           <t>Escalation</t>
         </is>
       </c>
-      <c r="B33" s="10" t="inlineStr">
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>Bot tự báo sếp / route reminder khi quá hạn</t>
         </is>
       </c>
-      <c r="C33" s="11" t="inlineStr">
+      <c r="C36" s="11" t="inlineStr">
         <is>
           <t>E3</t>
         </is>
       </c>
-      <c r="D33" s="11" t="inlineStr">
+      <c r="D36" s="11" t="inlineStr">
         <is>
           <t>Task từ group, assignee chưa join → reminder vào group</t>
         </is>
       </c>
-      <c r="E33" s="11" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>Task có Group ID + assignee không có Chat ID → reminder fallback vào group thay vì silent</t>
         </is>
       </c>
-      <c r="F33" s="12" t="inlineStr">
+      <c r="F36" s="12" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="G33" s="11" t="inlineStr">
+      <c r="G36" s="11" t="inlineStr">
         <is>
           <t>outbound vào source group</t>
         </is>
       </c>
-      <c r="H33" s="11" t="inlineStr">
+      <c r="H36" s="11" t="inlineStr">
         <is>
           <t>FIXED — _resolve_task_targets helper trong scheduler; route theo Group ID khi present</t>
         </is>

</xml_diff>

<commit_message>
feat(reminder): also post into source group when fire (auto-detect + report back)
When a reminder is created via @mention in a group ("@bot nhắc Long 5h
chiều mai họp"), the whole team saw the request — they should also see
the follow-up so the team knows the bot actually nhắc. Until now the fire
only DM'd the target + sent a private confirm to boss; the source group
stayed silent.

`reminder_agent.send_reminder` now sends a short "⏰ Vừa nhắc X: …" into
`source_chat_id` after the LLM-written DM to target, when source is set
and isn't already the dest/boss (no duplicate sends).

R3 scenario tightened to three destinations:
  - target DM
  - boss cc (already existed)
  - source group public notice (new behaviour)

Self-test reminder cluster: 6/6 pass.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/self_test_clusters.xlsx
+++ b/docs/self_test_clusters.xlsx
@@ -555,7 +555,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14 14:40</t>
+          <t>2026-05-14 15:38</t>
         </is>
       </c>
     </row>
@@ -944,12 +944,12 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Fire reminder bypass scheduler</t>
+          <t>Fire reminder có target + source group → 3 destinations</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>send_reminder(target_chat_id) trực tiếp → DM tới target</t>
+          <t>send_reminder(target_chat_id + source_chat_id) → target nhận DM + boss nhận cc + source group nhận public notice 'Vừa nhắc X: ...'</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
@@ -959,12 +959,12 @@
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
-          <t>outbound tới target_chat_id</t>
+          <t>3 outbound: target DM, boss cc, source group</t>
         </is>
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>FIXED — reminder_agent.send_reminder giờ post thêm notice vào source group khi reminder được tạo trong group context</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(reminder): R5/R6 — verify solo reminders never leak to group
The new "post into source group on fire" behaviour from the previous
commit only kicks in when `source_chat_id` is set, but the previous test
suite never explicitly verified that solo reminders (created in DM, no
source) STAY solo. Two new strict scenarios close that gap:

- R5 "DM-only self": target=None, source=None — fire must DM boss only.
  Asserts neither the group nor any third-party DM gets the reminder.
- R6 "DM-only boss → member": target=Long, source=None — fire must DM
  Long + cc boss, and the group must NOT receive any post.

Both PASS; confirms the source-group notify branch in send_reminder is
correctly gated on `source_chat_id` truthiness.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/self_test_clusters.xlsx
+++ b/docs/self_test_clusters.xlsx
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -555,7 +555,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14 15:38</t>
+          <t>2026-05-14 15:43</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>23</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>23</t>
         </is>
       </c>
     </row>
@@ -1011,39 +1011,71 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Reminder</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Tạo / fire / nhận diện nguồn reminder</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Fire DM-only self-reminder → chỉ boss</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Self-reminder trong DM (target=None, source=None) → fire chỉ DM boss; KHÔNG group, KHÔNG DM người khác</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>outbound chỉ tới boss conv</t>
+        </is>
+      </c>
+      <c r="H19" s="11" t="inlineStr">
+        <is>
+          <t>Đảm bảo nhắc lẻ không bị leak ra group / contact khác</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Reminder</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Khả năng auto-take note từ hội thoại tự nhiên</t>
+          <t>Tạo / fire / nhận diện nguồn reminder</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>R6</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Auto-append khi boss chia sẻ context cá nhân</t>
+          <t>Fire DM-only target reminder → DM target + boss, KHÔNG group</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>Boss nói 'gọi tôi là anh Đạt' → bot append_note / update_note</t>
+          <t>Boss DM tạo reminder cho Long (target có, source=None) → fire DM Long + cc boss; group KHÔNG có post</t>
         </is>
       </c>
       <c r="F20" s="12" t="inlineStr">
@@ -1053,12 +1085,12 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>tool append_note / update_note được gọi</t>
+          <t>outbound tới target DM + boss; group conv không có</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Bảo đảm boss DM riêng → fire không lén post vào group</t>
         </is>
       </c>
     </row>
@@ -1075,27 +1107,27 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>File-Link</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Bot xử lý file đính kèm và link YouTube/TikTok/báo</t>
+          <t>Khả năng auto-take note từ hội thoại tự nhiên</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>DM gửi file text + caption</t>
+          <t>Auto-append khi boss chia sẻ context cá nhân</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>Boss gửi .txt + 'tóm tắt' → bot phải đọc nội dung file (keyword đặc trưng zulipix/qorantek phải xuất hiện)</t>
+          <t>Boss nói 'gọi tôi là anh Đạt' → bot append_note / update_note</t>
         </is>
       </c>
       <c r="F22" s="12" t="inlineStr">
@@ -1105,56 +1137,24 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>bot reference keyword zulipix/qorantek từ file</t>
+          <t>tool append_note / update_note được gọi</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>FIXED — _ingest_text handler đọc text/plain (Zalo bridge thường drop mime)</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>File-Link</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>Bot xử lý file đính kèm và link YouTube/TikTok/báo</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="inlineStr">
-        <is>
-          <t>F2</t>
-        </is>
-      </c>
-      <c r="D23" s="11" t="inlineStr">
-        <is>
-          <t>DM paste link YouTube</t>
-        </is>
-      </c>
-      <c r="E23" s="11" t="inlineStr">
-        <is>
-          <t>Boss gửi YouTube link → bot fetch via oEmbed</t>
-        </is>
-      </c>
-      <c r="F23" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G23" s="11" t="inlineStr">
-        <is>
-          <t>tool fetch_url được gọi</t>
-        </is>
-      </c>
-      <c r="H23" s="11" t="inlineStr">
-        <is>
-          <t>FIXED — fetch_url tool mới + url_fetch_service hit YouTube oEmbed</t>
-        </is>
-      </c>
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
@@ -1169,17 +1169,17 @@
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>DM paste link TikTok</t>
+          <t>DM gửi file text + caption</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>Boss gửi TikTok link → bot fetch via oEmbed</t>
+          <t>Boss gửi .txt + 'tóm tắt' → bot phải đọc nội dung file (keyword đặc trưng zulipix/qorantek phải xuất hiện)</t>
         </is>
       </c>
       <c r="F24" s="12" t="inlineStr">
@@ -1189,12 +1189,12 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>tool fetch_url được gọi</t>
+          <t>bot reference keyword zulipix/qorantek từ file</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>FIXED — fetch_url tool</t>
+          <t>FIXED — _ingest_text handler đọc text/plain (Zalo bridge thường drop mime)</t>
         </is>
       </c>
     </row>
@@ -1211,17 +1211,17 @@
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>DM paste link bài báo (vnexpress)</t>
+          <t>DM paste link YouTube</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>Boss gửi link tin tức → bot fetch HTML + summary</t>
+          <t>Boss gửi YouTube link → bot fetch via oEmbed</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>Path generic HTML qua fetch_url (trước đây dùng web_search; giờ chính xác hơn)</t>
+          <t>FIXED — fetch_url tool mới + url_fetch_service hit YouTube oEmbed</t>
         </is>
       </c>
     </row>
@@ -1253,17 +1253,17 @@
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>F5</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Image attachment (PNG 32x32 đỏ)</t>
+          <t>DM paste link TikTok</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>Boss gửi ảnh + 'trong ảnh này có gì' → bot ingest, reply nhắc ảnh/màu</t>
+          <t>Boss gửi TikTok link → bot fetch via oEmbed</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
@@ -1273,49 +1273,81 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>reply nhắc tới ảnh / màu</t>
+          <t>tool fetch_url được gọi</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>File ingestion → LOCAL_IMAGE sentinel + OpenAI Vision</t>
+          <t>FIXED — fetch_url tool</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>File-Link</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Bot xử lý file đính kèm và link YouTube/TikTok/báo</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>DM paste link bài báo (vnexpress)</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>Boss gửi link tin tức → bot fetch HTML + summary</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G27" s="11" t="inlineStr">
+        <is>
+          <t>tool fetch_url được gọi</t>
+        </is>
+      </c>
+      <c r="H27" s="11" t="inlineStr">
+        <is>
+          <t>Path generic HTML qua fetch_url (trước đây dùng web_search; giờ chính xác hơn)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Onboard</t>
+          <t>File-Link</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Hỏi boss / xin phép khi có người mới</t>
+          <t>Bot xử lý file đính kèm và link YouTube/TikTok/báo</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>O1</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>New-member event trong group → bot phải hỏi boss</t>
+          <t>Image attachment (PNG 32x32 đỏ)</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>Người mới vào group đã onboarded → bot proactive DM boss hỏi role</t>
+          <t>Boss gửi ảnh + 'trong ảnh này có gì' → bot ingest, reply nhắc ảnh/màu</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
@@ -1325,56 +1357,24 @@
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>outbound tới boss có tên 'Người Mới'</t>
+          <t>reply nhắc tới ảnh / màu</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>FIXED — _notify_boss_new_members trong secretary_agent.handle_message (qua _messenger_for nên route đúng channel boss)</t>
+          <t>File ingestion → LOCAL_IMAGE sentinel + OpenAI Vision</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>Onboard</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>Hỏi boss / xin phép khi có người mới</t>
-        </is>
-      </c>
-      <c r="C29" s="11" t="inlineStr">
-        <is>
-          <t>O2</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="inlineStr">
-        <is>
-          <t>Boss duyệt pending member</t>
-        </is>
-      </c>
-      <c r="E29" s="11" t="inlineStr">
-        <is>
-          <t>Pre-insert pending membership → boss DM 'duyệt' → approve_join → membership active</t>
-        </is>
-      </c>
-      <c r="F29" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G29" s="11" t="inlineStr">
-        <is>
-          <t>tool approve_join + membership.status='active'</t>
-        </is>
-      </c>
-      <c r="H29" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
@@ -1389,17 +1389,17 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>O3</t>
+          <t>O1</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Stranger gọi request_join → pending row + boss được DM</t>
+          <t>New-member event trong group → bot phải hỏi boss</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>Stranger gọi service request_join → membership pending + boss nhận outbound</t>
+          <t>Người mới vào group đã onboarded → bot proactive DM boss hỏi role</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
@@ -1409,49 +1409,81 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>membership status=pending + outbound to boss conv</t>
+          <t>outbound tới boss có tên 'Người Mới'</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>Test phần TRƯỚC của join flow</t>
+          <t>FIXED — _notify_boss_new_members trong secretary_agent.handle_message (qua _messenger_for nên route đúng channel boss)</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>Onboard</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Hỏi boss / xin phép khi có người mới</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>O2</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>Boss duyệt pending member</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>Pre-insert pending membership → boss DM 'duyệt' → approve_join → membership active</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>tool approve_join + membership.status='active'</t>
+        </is>
+      </c>
+      <c r="H31" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>Escalation</t>
+          <t>Onboard</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>Bot tự báo sếp / route reminder khi quá hạn</t>
+          <t>Hỏi boss / xin phép khi có người mới</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>O3</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Task overdue (DM context) → assignee DM + boss report</t>
+          <t>Stranger gọi request_join → pending row + boss được DM</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>Task không có Group ID + assignee có Chat ID → reminder DM tới assignee + boss nhận report</t>
+          <t>Stranger gọi service request_join → membership pending + boss nhận outbound</t>
         </is>
       </c>
       <c r="F32" s="12" t="inlineStr">
@@ -1461,56 +1493,24 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>outbound tới assignee DM + boss conv</t>
+          <t>membership status=pending + outbound to boss conv</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Test phần TRƯỚC của join flow</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="9" t="inlineStr">
-        <is>
-          <t>Escalation</t>
-        </is>
-      </c>
-      <c r="B33" s="10" t="inlineStr">
-        <is>
-          <t>Bot tự báo sếp / route reminder khi quá hạn</t>
-        </is>
-      </c>
-      <c r="C33" s="11" t="inlineStr">
-        <is>
-          <t>E2</t>
-        </is>
-      </c>
-      <c r="D33" s="11" t="inlineStr">
-        <is>
-          <t>Member bị nhắc deadline không reply → bot báo sếp</t>
-        </is>
-      </c>
-      <c r="E33" s="11" t="inlineStr">
-        <is>
-          <t>Reminder fire 4h trước, target im lặng → _check_no_reply_reminders → bot DM boss</t>
-        </is>
-      </c>
-      <c r="F33" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G33" s="11" t="inlineStr">
-        <is>
-          <t>outbound nhắc boss về Long + escalated=1</t>
-        </is>
-      </c>
-      <c r="H33" s="11" t="inlineStr">
-        <is>
-          <t>FIXED — _check_no_reply_reminders scheduler tick mới (30 phút) + outbound_messages.escalated column</t>
-        </is>
-      </c>
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
@@ -1525,17 +1525,17 @@
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Task từ group, assignee chưa join → reminder vào group</t>
+          <t>Task overdue (DM context) → assignee DM + boss report</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>Task có Group ID + assignee không có Chat ID → reminder fallback vào group</t>
+          <t>Task không có Group ID + assignee có Chat ID → reminder DM tới assignee + boss nhận report</t>
         </is>
       </c>
       <c r="F34" s="12" t="inlineStr">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>outbound vào source group</t>
+          <t>outbound tới assignee DM + boss conv</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -1555,52 +1555,136 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr"/>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>Bot tự báo sếp / route reminder khi quá hạn</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D35" s="11" t="inlineStr">
+        <is>
+          <t>Member bị nhắc deadline không reply → bot báo sếp</t>
+        </is>
+      </c>
+      <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>Reminder fire 4h trước, target im lặng → _check_no_reply_reminders → bot DM boss</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G35" s="11" t="inlineStr">
+        <is>
+          <t>outbound nhắc boss về Long + escalated=1</t>
+        </is>
+      </c>
+      <c r="H35" s="11" t="inlineStr">
+        <is>
+          <t>FIXED — _check_no_reply_reminders scheduler tick mới (30 phút) + outbound_messages.escalated column</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>Bot tự báo sếp / route reminder khi quá hạn</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t>Task từ group, assignee chưa join → reminder vào group</t>
+        </is>
+      </c>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>Task có Group ID + assignee không có Chat ID → reminder fallback vào group</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="inlineStr">
+        <is>
+          <t>outbound vào source group</t>
+        </is>
+      </c>
+      <c r="H36" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
           <t>Channel</t>
         </is>
       </c>
-      <c r="B36" s="10" t="inlineStr">
+      <c r="B38" s="10" t="inlineStr">
         <is>
           <t>Cross-channel isolation per boss</t>
         </is>
       </c>
-      <c r="C36" s="11" t="inlineStr">
+      <c r="C38" s="11" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="D36" s="11" t="inlineStr">
+      <c r="D38" s="11" t="inlineStr">
         <is>
           <t>Boss Zalo + Telegram-only assignee → reminder vào group, KHÔNG DM cross-channel</t>
         </is>
       </c>
-      <c r="E36" s="11" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>Boss có primary_channel='zalo', assignee chỉ có Telegram identity → reminder PHẢI vào group, KHÔNG được DM Long qua Telegram</t>
         </is>
       </c>
-      <c r="F36" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G36" s="11" t="inlineStr">
+      <c r="F38" s="12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G38" s="11" t="inlineStr">
         <is>
           <t>outbound vào group + KHÔNG outbound vào Long DM</t>
         </is>
       </c>
-      <c r="H36" s="11" t="inlineStr">
+      <c r="H38" s="11" t="inlineStr">
         <is>
           <t>FIXED — bosses.primary_channel column + is_target_on_boss_channel filter trong _resolve_task_targets</t>
         </is>

</xml_diff>

<commit_message>
docs(self-test): trim CSV — drop redundant cluster_purpose + merge intent into name
The CSV had ballooned: cluster_purpose repeated identical text on every
row of a cluster, case_intent restated what case_name already says, and
half the notes column was just "-" placeholders. Reading it was harder
than reading the live xlsx.

New layout (6 cols):
  cluster | case_id | scenario | status | evidence | notes

- cluster_purpose dropped (cluster name self-explains)
- case_name + case_intent merged into one scenario column
- notes only carry actual info now (fix references / why), no "-" filler

CSV: 4669 → 3168 bytes (-32%). xlsx generator updated to the new column
indices; summary block + freeze pane preserved.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/self_test_clusters.xlsx
+++ b/docs/self_test_clusters.xlsx
@@ -124,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -151,9 +151,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -527,17 +524,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="64" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="56" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="56" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -555,7 +550,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14 16:11</t>
+          <t>2026-05-14 16:30</t>
         </is>
       </c>
     </row>
@@ -630,35 +625,25 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>cluster_purpose</t>
+          <t>case_id</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>case_id</t>
+          <t>scenario</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>case_name</t>
+          <t>status</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>case_intent</t>
+          <t>evidence</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>evidence</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -672,39 +657,25 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Boss tạo / liệt kê / cập nhật task qua DM hoặc group</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="inlineStr">
-        <is>
           <t>T1</t>
         </is>
       </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>DM tạo task — bot gọi create_task</t>
+        </is>
+      </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>DM tạo task</t>
-        </is>
-      </c>
-      <c r="E10" s="11" t="inlineStr">
-        <is>
-          <t>Boss DM bot 'tạo task ...' → bot gọi create_task</t>
-        </is>
-      </c>
-      <c r="F10" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G10" s="11" t="inlineStr">
-        <is>
-          <t>tool create_task được gọi</t>
-        </is>
-      </c>
-      <c r="H10" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>create_task tool called</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -714,39 +685,25 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Boss tạo / liệt kê / cập nhật task qua DM hoặc group</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="inlineStr">
-        <is>
           <t>T2</t>
         </is>
       </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>DM liệt kê task — bot gọi list_tasks</t>
+        </is>
+      </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>DM liệt kê task</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="inlineStr">
-        <is>
-          <t>Boss DM 'cho xem danh sách task' → bot gọi list_tasks</t>
-        </is>
-      </c>
-      <c r="F11" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G11" s="11" t="inlineStr">
-        <is>
-          <t>tool list_tasks được gọi</t>
-        </is>
-      </c>
-      <c r="H11" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>list_tasks tool called</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -756,39 +713,25 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Boss tạo / liệt kê / cập nhật task qua DM hoặc group</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="inlineStr">
-        <is>
           <t>T3a</t>
         </is>
       </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Group @mention giao task — Telegram assignee (id numeric)</t>
+        </is>
+      </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Group @mention giao task — Telegram assignee</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="inlineStr">
-        <is>
-          <t>Trong group, boss @bot 'giao Long task' (Chat ID Telegram numeric) → resolve được id, create_task không crash</t>
-        </is>
-      </c>
-      <c r="F12" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G12" s="11" t="inlineStr">
-        <is>
-          <t>tool create_task không lỗi</t>
-        </is>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>create_task không lỗi</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -798,39 +741,25 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Boss tạo / liệt kê / cập nhật task qua DM hoặc group</t>
-        </is>
-      </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
           <t>T3b</t>
         </is>
       </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Group @mention giao task — Zalo assignee (id alphanum)</t>
+        </is>
+      </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Group @mention giao task — Zalo assignee</t>
-        </is>
-      </c>
-      <c r="E13" s="11" t="inlineStr">
-        <is>
-          <t>Trong group, boss @bot 'giao Hùng task' (Chat ID Zalo alphanum) → resolve được id, create_task không crash</t>
-        </is>
-      </c>
-      <c r="F13" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G13" s="11" t="inlineStr">
-        <is>
-          <t>tool create_task không lỗi</t>
-        </is>
-      </c>
-      <c r="H13" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>create_task không lỗi</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
@@ -839,8 +768,6 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -850,39 +777,25 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Tạo / fire / nhận diện nguồn reminder</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
           <t>R1</t>
         </is>
       </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>DM self-reminder</t>
+        </is>
+      </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>DM: self-reminder</t>
-        </is>
-      </c>
-      <c r="E15" s="11" t="inlineStr">
-        <is>
-          <t>Boss DM 'nhắc tôi ...' → tool create_reminder với target=boss</t>
-        </is>
-      </c>
-      <c r="F15" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G15" s="11" t="inlineStr">
-        <is>
-          <t>tool create_reminder được gọi</t>
-        </is>
-      </c>
-      <c r="H15" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>create_reminder called</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -892,39 +805,25 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Tạo / fire / nhận diện nguồn reminder</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="inlineStr">
-        <is>
           <t>R2</t>
         </is>
       </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Group @mention nhắc 1 member</t>
+        </is>
+      </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Group @mention nhắc 1 member</t>
-        </is>
-      </c>
-      <c r="E16" s="11" t="inlineStr">
-        <is>
-          <t>Trong group, boss @bot 'nhắc Long' → create_reminder với target=member, source_chat_id=group</t>
-        </is>
-      </c>
-      <c r="F16" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G16" s="11" t="inlineStr">
-        <is>
-          <t>tool create_reminder được gọi</t>
-        </is>
-      </c>
-      <c r="H16" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>create_reminder called với target + source_chat_id</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -934,37 +833,27 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Tạo / fire / nhận diện nguồn reminder</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
           <t>R3</t>
         </is>
       </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Fire reminder target + source group → 3 destinations</t>
+        </is>
+      </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Fire reminder có target + source group → 3 destinations</t>
-        </is>
-      </c>
-      <c r="E17" s="11" t="inlineStr">
-        <is>
-          <t>send_reminder(target_chat_id + source_chat_id) → target nhận DM + boss nhận cc + source group nhận public notice 'Vừa nhắc X: ...'</t>
-        </is>
-      </c>
-      <c r="F17" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G17" s="11" t="inlineStr">
-        <is>
-          <t>3 outbound: target DM, boss cc, source group</t>
-        </is>
-      </c>
-      <c r="H17" s="11" t="inlineStr">
-        <is>
-          <t>FIXED — reminder_agent.send_reminder giờ post thêm notice vào source group khi reminder được tạo trong group context</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>target DM + boss cc + source group public notice</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>reminder_agent post thêm vào source_chat_id</t>
         </is>
       </c>
     </row>
@@ -976,39 +865,25 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Tạo / fire / nhận diện nguồn reminder</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
           <t>R4</t>
         </is>
       </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Fire reminder source-only (không target) → vào source group</t>
+        </is>
+      </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Fire reminder source-only</t>
-        </is>
-      </c>
-      <c r="E18" s="11" t="inlineStr">
-        <is>
-          <t>Reminder không có target_chat_id, có source_chat_id → outbound vào source group thay vì DM boss</t>
-        </is>
-      </c>
-      <c r="F18" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G18" s="11" t="inlineStr">
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>outbound vào source group</t>
         </is>
       </c>
-      <c r="H18" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="F18" s="10" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1018,39 +893,25 @@
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Tạo / fire / nhận diện nguồn reminder</t>
-        </is>
-      </c>
-      <c r="C19" s="11" t="inlineStr">
-        <is>
           <t>R5</t>
         </is>
       </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Fire DM-only self-reminder → chỉ boss</t>
+        </is>
+      </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Fire DM-only self-reminder → chỉ boss</t>
-        </is>
-      </c>
-      <c r="E19" s="11" t="inlineStr">
-        <is>
-          <t>Self-reminder trong DM (target=None, source=None) → fire chỉ DM boss; KHÔNG group, KHÔNG DM người khác</t>
-        </is>
-      </c>
-      <c r="F19" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G19" s="11" t="inlineStr">
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
         <is>
           <t>outbound chỉ tới boss conv</t>
         </is>
       </c>
-      <c r="H19" s="11" t="inlineStr">
-        <is>
-          <t>Đảm bảo nhắc lẻ không bị leak ra group / contact khác</t>
-        </is>
-      </c>
+      <c r="F19" s="10" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
@@ -1060,39 +921,25 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Tạo / fire / nhận diện nguồn reminder</t>
-        </is>
-      </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
           <t>R6</t>
         </is>
       </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>Fire DM-only target reminder → DM target + boss, KHÔNG group</t>
+        </is>
+      </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Fire DM-only target reminder → DM target + boss, KHÔNG group</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>Boss DM tạo reminder cho Long (target có, source=None) → fire DM Long + cc boss; group KHÔNG có post</t>
-        </is>
-      </c>
-      <c r="F20" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G20" s="11" t="inlineStr">
-        <is>
-          <t>outbound tới target DM + boss; group conv không có</t>
-        </is>
-      </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>Bảo đảm boss DM riêng → fire không lén post vào group</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>target DM + boss cc; group conv không có</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
@@ -1101,8 +948,6 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
@@ -1112,39 +957,25 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Khả năng auto-take note từ hội thoại tự nhiên</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="inlineStr">
-        <is>
           <t>N1</t>
         </is>
       </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>Auto-append note khi boss chia sẻ context cá nhân</t>
+        </is>
+      </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Auto-append khi boss chia sẻ context cá nhân</t>
-        </is>
-      </c>
-      <c r="E22" s="11" t="inlineStr">
-        <is>
-          <t>Boss nói 'gọi tôi là anh Đạt' → bot append_note / update_note</t>
-        </is>
-      </c>
-      <c r="F22" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G22" s="11" t="inlineStr">
-        <is>
-          <t>tool append_note / update_note được gọi</t>
-        </is>
-      </c>
-      <c r="H22" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>append_note / update_note called</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
@@ -1153,8 +984,6 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
@@ -1164,37 +993,27 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>Bot xử lý file đính kèm và link YouTube/TikTok/báo</t>
-        </is>
-      </c>
-      <c r="C24" s="11" t="inlineStr">
-        <is>
           <t>F1</t>
         </is>
       </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>DM gửi file .txt + caption — bot đọc nội dung</t>
+        </is>
+      </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>DM gửi file text + caption</t>
-        </is>
-      </c>
-      <c r="E24" s="11" t="inlineStr">
-        <is>
-          <t>Boss gửi .txt + 'tóm tắt' → bot phải đọc nội dung file (keyword đặc trưng zulipix/qorantek phải xuất hiện)</t>
-        </is>
-      </c>
-      <c r="F24" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G24" s="11" t="inlineStr">
-        <is>
-          <t>bot reference keyword zulipix/qorantek từ file</t>
-        </is>
-      </c>
-      <c r="H24" s="11" t="inlineStr">
-        <is>
-          <t>FIXED — _ingest_text handler đọc text/plain (Zalo bridge thường drop mime)</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>reply reference keyword đặc trưng từ file</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>_ingest_text handler cho text/plain</t>
         </is>
       </c>
     </row>
@@ -1206,37 +1025,27 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>Bot xử lý file đính kèm và link YouTube/TikTok/báo</t>
-        </is>
-      </c>
-      <c r="C25" s="11" t="inlineStr">
-        <is>
           <t>F2</t>
         </is>
       </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>DM paste link YouTube — bot fetch metadata + transcript</t>
+        </is>
+      </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>DM paste link YouTube</t>
-        </is>
-      </c>
-      <c r="E25" s="11" t="inlineStr">
-        <is>
-          <t>Boss gửi YouTube link → bot fetch via oEmbed</t>
-        </is>
-      </c>
-      <c r="F25" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G25" s="11" t="inlineStr">
-        <is>
-          <t>tool fetch_url được gọi</t>
-        </is>
-      </c>
-      <c r="H25" s="11" t="inlineStr">
-        <is>
-          <t>FIXED — fetch_url tool mới + url_fetch_service hit YouTube oEmbed</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>fetch_url called</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>fetch_url tool + url_fetch_service oEmbed + youtube-transcript-api</t>
         </is>
       </c>
     </row>
@@ -1248,37 +1057,27 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Bot xử lý file đính kèm và link YouTube/TikTok/báo</t>
-        </is>
-      </c>
-      <c r="C26" s="11" t="inlineStr">
-        <is>
           <t>F3</t>
         </is>
       </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>DM paste link TikTok — bot fetch oEmbed + yt-dlp metadata</t>
+        </is>
+      </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>DM paste link TikTok</t>
-        </is>
-      </c>
-      <c r="E26" s="11" t="inlineStr">
-        <is>
-          <t>Boss gửi TikTok link → bot fetch via oEmbed</t>
-        </is>
-      </c>
-      <c r="F26" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G26" s="11" t="inlineStr">
-        <is>
-          <t>tool fetch_url được gọi</t>
-        </is>
-      </c>
-      <c r="H26" s="11" t="inlineStr">
-        <is>
-          <t>FIXED — fetch_url tool</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>fetch_url called</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>fetch_url tool — caption/uploader/duration/views</t>
         </is>
       </c>
     </row>
@@ -1290,39 +1089,25 @@
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>Bot xử lý file đính kèm và link YouTube/TikTok/báo</t>
-        </is>
-      </c>
-      <c r="C27" s="11" t="inlineStr">
-        <is>
           <t>F4</t>
         </is>
       </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>DM paste link bài báo — bot fetch HTML summary</t>
+        </is>
+      </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>DM paste link bài báo (vnexpress)</t>
-        </is>
-      </c>
-      <c r="E27" s="11" t="inlineStr">
-        <is>
-          <t>Boss gửi link tin tức → bot fetch HTML + summary</t>
-        </is>
-      </c>
-      <c r="F27" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G27" s="11" t="inlineStr">
-        <is>
-          <t>tool fetch_url được gọi</t>
-        </is>
-      </c>
-      <c r="H27" s="11" t="inlineStr">
-        <is>
-          <t>Path generic HTML qua fetch_url (trước đây dùng web_search; giờ chính xác hơn)</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>fetch_url called</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
@@ -1332,37 +1117,27 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Bot xử lý file đính kèm và link YouTube/TikTok/báo</t>
-        </is>
-      </c>
-      <c r="C28" s="11" t="inlineStr">
-        <is>
           <t>F5</t>
         </is>
       </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>Image attachment (PNG) — bot nhận diện ảnh</t>
+        </is>
+      </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Image attachment (PNG 32x32 đỏ)</t>
-        </is>
-      </c>
-      <c r="E28" s="11" t="inlineStr">
-        <is>
-          <t>Boss gửi ảnh + 'trong ảnh này có gì' → bot ingest, reply nhắc ảnh/màu</t>
-        </is>
-      </c>
-      <c r="F28" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G28" s="11" t="inlineStr">
-        <is>
-          <t>reply nhắc tới ảnh / màu</t>
-        </is>
-      </c>
-      <c r="H28" s="11" t="inlineStr">
-        <is>
-          <t>File ingestion → LOCAL_IMAGE sentinel + OpenAI Vision</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>reply nhắc tới ảnh/màu</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>LOCAL_IMAGE sentinel + OpenAI Vision</t>
         </is>
       </c>
     </row>
@@ -1373,8 +1148,6 @@
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
@@ -1384,37 +1157,27 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Hỏi boss / xin phép khi có người mới</t>
-        </is>
-      </c>
-      <c r="C30" s="11" t="inlineStr">
-        <is>
           <t>O1</t>
         </is>
       </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>New-member event trong group → bot proactive DM boss</t>
+        </is>
+      </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>New-member event trong group → bot phải hỏi boss</t>
-        </is>
-      </c>
-      <c r="E30" s="11" t="inlineStr">
-        <is>
-          <t>Người mới vào group đã onboarded → bot proactive DM boss hỏi role</t>
-        </is>
-      </c>
-      <c r="F30" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G30" s="11" t="inlineStr">
-        <is>
-          <t>outbound tới boss có tên 'Người Mới'</t>
-        </is>
-      </c>
-      <c r="H30" s="11" t="inlineStr">
-        <is>
-          <t>FIXED — _notify_boss_new_members trong secretary_agent.handle_message (qua _messenger_for nên route đúng channel boss)</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>outbound tới boss có tên người mới</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>_notify_boss_new_members route qua channel của boss</t>
         </is>
       </c>
     </row>
@@ -1426,37 +1189,27 @@
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>Hỏi boss / xin phép khi có người mới</t>
-        </is>
-      </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
           <t>O2</t>
         </is>
       </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>Boss duyệt + stranger được báo qua channel của họ</t>
+        </is>
+      </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>Boss duyệt + stranger được báo qua channel của họ</t>
-        </is>
-      </c>
-      <c r="E31" s="11" t="inlineStr">
-        <is>
-          <t>Boss DM duyệt → approve_join → membership active + stranger nhận outbound qua channel của stranger</t>
-        </is>
-      </c>
-      <c r="F31" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G31" s="11" t="inlineStr">
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
         <is>
           <t>approve_join + membership active + outbound vào stranger conv</t>
         </is>
       </c>
-      <c r="H31" s="11" t="inlineStr">
-        <is>
-          <t>FIXED — approve_join notify stranger qua _messenger_for</t>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>approve_join giờ notify stranger</t>
         </is>
       </c>
     </row>
@@ -1468,39 +1221,25 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>Hỏi boss / xin phép khi có người mới</t>
-        </is>
-      </c>
-      <c r="C32" s="11" t="inlineStr">
-        <is>
           <t>O3</t>
         </is>
       </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>Stranger gọi request_join → pending row + boss DM</t>
+        </is>
+      </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Stranger gọi request_join → pending row + boss được DM</t>
-        </is>
-      </c>
-      <c r="E32" s="11" t="inlineStr">
-        <is>
-          <t>Stranger gọi service request_join → membership pending + boss nhận outbound</t>
-        </is>
-      </c>
-      <c r="F32" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G32" s="11" t="inlineStr">
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
         <is>
           <t>membership status=pending + outbound to boss conv</t>
         </is>
       </c>
-      <c r="H32" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="F32" s="10" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
@@ -1510,37 +1249,27 @@
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Hỏi boss / xin phép khi có người mới</t>
-        </is>
-      </c>
-      <c r="C33" s="11" t="inlineStr">
-        <is>
           <t>O4</t>
         </is>
       </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>Listing isolation: Zalo stranger không thấy boss Telegram</t>
+        </is>
+      </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>Listing isolation: Zalo stranger không thấy boss Telegram</t>
-        </is>
-      </c>
-      <c r="E33" s="11" t="inlineStr">
-        <is>
-          <t>handle_join_inquiry từ Zalo conv: response KHÔNG chứa tên boss Telegram. Từ Telegram conv: response CÓ.</t>
-        </is>
-      </c>
-      <c r="F33" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G33" s="11" t="inlineStr">
-        <is>
-          <t>Zalo listing không chứa 'Linh'; Telegram listing có 'Linh'</t>
-        </is>
-      </c>
-      <c r="H33" s="11" t="inlineStr">
-        <is>
-          <t>FIXED — _filter_bosses_for_channel strict isolation: stranger Zalo không thể chọn boss Telegram ngay từ tầng listing. Bosses NULL primary_channel cũng bị hide.</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>Zalo listing không chứa 'Linh'; Telegram listing có</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>_filter_bosses_for_channel strict — NULL primary_channel cũng hidden</t>
         </is>
       </c>
     </row>
@@ -1551,8 +1280,6 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
@@ -1562,39 +1289,25 @@
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Bot tự báo sếp / route reminder khi quá hạn</t>
-        </is>
-      </c>
-      <c r="C35" s="11" t="inlineStr">
-        <is>
           <t>E1</t>
         </is>
       </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>Task overdue (DM context) → assignee DM + boss report</t>
+        </is>
+      </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>Task overdue (DM context) → assignee DM + boss report</t>
-        </is>
-      </c>
-      <c r="E35" s="11" t="inlineStr">
-        <is>
-          <t>Task không có Group ID + assignee có Chat ID → reminder DM tới assignee + boss nhận report</t>
-        </is>
-      </c>
-      <c r="F35" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G35" s="11" t="inlineStr">
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
         <is>
           <t>outbound tới assignee DM + boss conv</t>
         </is>
       </c>
-      <c r="H35" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="F35" s="10" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
@@ -1604,37 +1317,27 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>Bot tự báo sếp / route reminder khi quá hạn</t>
-        </is>
-      </c>
-      <c r="C36" s="11" t="inlineStr">
-        <is>
           <t>E2</t>
         </is>
       </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>Member nhắc deadline không reply → bot báo sếp</t>
+        </is>
+      </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Member bị nhắc deadline không reply → bot báo sếp</t>
-        </is>
-      </c>
-      <c r="E36" s="11" t="inlineStr">
-        <is>
-          <t>Reminder fire 4h trước, target im lặng → _check_no_reply_reminders → bot DM boss</t>
-        </is>
-      </c>
-      <c r="F36" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G36" s="11" t="inlineStr">
-        <is>
-          <t>outbound nhắc boss về Long + escalated=1</t>
-        </is>
-      </c>
-      <c r="H36" s="11" t="inlineStr">
-        <is>
-          <t>FIXED — _check_no_reply_reminders scheduler tick mới (30 phút) + outbound_messages.escalated column</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>outbound nhắc boss + escalated=1</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="inlineStr">
+        <is>
+          <t>_check_no_reply_reminders tick 30min + outbound_messages.escalated</t>
         </is>
       </c>
     </row>
@@ -1646,39 +1349,25 @@
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>Bot tự báo sếp / route reminder khi quá hạn</t>
-        </is>
-      </c>
-      <c r="C37" s="11" t="inlineStr">
-        <is>
           <t>E3</t>
         </is>
       </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>Task từ group, assignee chưa join → reminder vào group</t>
+        </is>
+      </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>Task từ group, assignee chưa join → reminder vào group</t>
-        </is>
-      </c>
-      <c r="E37" s="11" t="inlineStr">
-        <is>
-          <t>Task có Group ID + assignee không có Chat ID → reminder fallback vào group</t>
-        </is>
-      </c>
-      <c r="F37" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G37" s="11" t="inlineStr">
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E37" s="10" t="inlineStr">
         <is>
           <t>outbound vào source group</t>
         </is>
       </c>
-      <c r="H37" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="F37" s="10" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
@@ -1687,8 +1376,6 @@
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
@@ -1698,43 +1385,33 @@
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>Cross-channel isolation per boss</t>
-        </is>
-      </c>
-      <c r="C39" s="11" t="inlineStr">
-        <is>
           <t>C1</t>
         </is>
       </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>Boss Zalo + Telegram-only assignee → reminder vào group, KHÔNG DM cross-channel</t>
+        </is>
+      </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>Boss Zalo + Telegram-only assignee → reminder vào group, KHÔNG DM cross-channel</t>
-        </is>
-      </c>
-      <c r="E39" s="11" t="inlineStr">
-        <is>
-          <t>Boss có primary_channel='zalo', assignee chỉ có Telegram identity → reminder PHẢI vào group, KHÔNG được DM Long qua Telegram</t>
-        </is>
-      </c>
-      <c r="F39" s="12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G39" s="11" t="inlineStr">
-        <is>
-          <t>outbound vào group + KHÔNG outbound vào Long DM</t>
-        </is>
-      </c>
-      <c r="H39" s="11" t="inlineStr">
-        <is>
-          <t>FIXED — bosses.primary_channel column + is_target_on_boss_channel filter trong _resolve_task_targets</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
+        <is>
+          <t>outbound vào group; KHÔNG outbound vào Long DM</t>
+        </is>
+      </c>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>bosses.primary_channel + is_target_on_boss_channel filter</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>